<commit_message>
pending bulk upload in create records and footer pressure value input box
</commit_message>
<xml_diff>
--- a/client/public/RecordsTemplate/RecordsTemplate.xlsx
+++ b/client/public/RecordsTemplate/RecordsTemplate.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
   <si>
     <t>s.no</t>
   </si>
@@ -100,6 +100,9 @@
   </si>
   <si>
     <t>Monel 400</t>
+  </si>
+  <si>
+    <t>traceability_no</t>
   </si>
 </sst>
 </file>
@@ -426,16 +429,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:P2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="32.77734375" customWidth="1"/>
-    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="17" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="15.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -446,46 +449,49 @@
         <v>1</v>
       </c>
       <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
         <v>2</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>3</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>4</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>5</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>6</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>7</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>8</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>9</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>10</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>11</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>12</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>13</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:16" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
@@ -495,43 +501,46 @@
       <c r="C2">
         <v>529890</v>
       </c>
-      <c r="D2" t="s">
+      <c r="D2">
+        <v>784</v>
+      </c>
+      <c r="E2" t="s">
         <v>17</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>18</v>
       </c>
-      <c r="F2">
+      <c r="G2">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="H2">
+      <c r="I2">
         <v>0.48930000000000001</v>
       </c>
-      <c r="I2">
+      <c r="J2">
         <v>0.48899999999999999</v>
       </c>
-      <c r="J2">
+      <c r="K2">
         <v>0.34300000000000003</v>
       </c>
-      <c r="K2">
+      <c r="L2">
         <v>0.434</v>
       </c>
-      <c r="L2">
+      <c r="M2">
         <v>0.34399999999999997</v>
       </c>
-      <c r="M2">
+      <c r="N2">
         <v>0.43</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>0.34399999999999997</v>
       </c>
-      <c r="O2">
+      <c r="P2">
         <v>0.34300000000000003</v>
       </c>
-      <c r="P2">
+      <c r="Q2">
         <v>0.434</v>
       </c>
     </row>

</xml_diff>

<commit_message>
dashboard updated and inspection & compliance certificate process completed
</commit_message>
<xml_diff>
--- a/client/public/RecordsTemplate/RecordsTemplate.xlsx
+++ b/client/public/RecordsTemplate/RecordsTemplate.xlsx
@@ -5,7 +5,7 @@
   <workbookPr defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\ExcelDataTransfer\client\public\RecordsTemplate\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sanjay\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="30">
   <si>
     <t>s.no</t>
   </si>
@@ -103,6 +103,18 @@
   </si>
   <si>
     <t>traceability_no</t>
+  </si>
+  <si>
+    <t>supplier_no</t>
+  </si>
+  <si>
+    <t>supplier_name</t>
+  </si>
+  <si>
+    <t>sup390</t>
+  </si>
+  <si>
+    <t>raja</t>
   </si>
 </sst>
 </file>
@@ -429,16 +441,16 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="32.77734375" customWidth="1"/>
-    <col min="6" max="6" width="14" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="4" width="32.77734375" customWidth="1"/>
+    <col min="8" max="8" width="14" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="17" bestFit="1" customWidth="1"/>
+    <col min="29" max="29" width="15.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -446,101 +458,113 @@
         <v>19</v>
       </c>
       <c r="C1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
       </c>
-      <c r="D1" t="s">
+      <c r="F1" t="s">
         <v>25</v>
       </c>
-      <c r="E1" t="s">
+      <c r="G1" t="s">
         <v>2</v>
       </c>
-      <c r="F1" t="s">
+      <c r="H1" t="s">
         <v>3</v>
       </c>
-      <c r="G1" t="s">
+      <c r="I1" t="s">
         <v>4</v>
       </c>
-      <c r="H1" t="s">
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="J1" t="s">
+      <c r="L1" t="s">
         <v>7</v>
       </c>
-      <c r="K1" t="s">
+      <c r="M1" t="s">
         <v>8</v>
       </c>
-      <c r="L1" t="s">
+      <c r="N1" t="s">
         <v>9</v>
       </c>
-      <c r="M1" t="s">
+      <c r="O1" t="s">
         <v>10</v>
       </c>
-      <c r="N1" t="s">
+      <c r="P1" t="s">
         <v>11</v>
       </c>
-      <c r="O1" t="s">
+      <c r="Q1" t="s">
         <v>12</v>
       </c>
-      <c r="P1" t="s">
+      <c r="R1" t="s">
         <v>13</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="S1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>29</v>
+      </c>
+      <c r="E2">
         <v>529890</v>
       </c>
-      <c r="D2">
+      <c r="F2">
         <v>784</v>
       </c>
-      <c r="E2" t="s">
+      <c r="G2" t="s">
         <v>17</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H2" t="s">
         <v>18</v>
       </c>
-      <c r="G2">
+      <c r="I2">
         <v>4.0000000000000001E-3</v>
       </c>
-      <c r="H2">
+      <c r="J2">
         <v>3.3999999999999998E-3</v>
       </c>
-      <c r="I2">
+      <c r="K2">
         <v>0.48930000000000001</v>
       </c>
-      <c r="J2">
+      <c r="L2">
         <v>0.48899999999999999</v>
       </c>
-      <c r="K2">
+      <c r="M2">
         <v>0.34300000000000003</v>
       </c>
-      <c r="L2">
+      <c r="N2">
         <v>0.434</v>
-      </c>
-      <c r="M2">
-        <v>0.34399999999999997</v>
-      </c>
-      <c r="N2">
-        <v>0.43</v>
       </c>
       <c r="O2">
         <v>0.34399999999999997</v>
       </c>
       <c r="P2">
+        <v>0.43</v>
+      </c>
+      <c r="Q2">
+        <v>0.34399999999999997</v>
+      </c>
+      <c r="R2">
         <v>0.34300000000000003</v>
       </c>
-      <c r="Q2">
+      <c r="S2">
         <v>0.434</v>
       </c>
     </row>

</xml_diff>